<commit_message>
Add pseudocode and flowchart for authentication automation
</commit_message>
<xml_diff>
--- a/test_case_and_bug_reporting/Test_Case_and_Bug_Reporting.xlsx
+++ b/test_case_and_bug_reporting/Test_Case_and_Bug_Reporting.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\QA_Test_Dummy\TugasQA_Rahardian_Era_Muliawan\test_case_and_bug_reporting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12B499F0-6726-47CC-950B-7189C8E98668}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D477776-D848-47A5-AAA9-8C61AB5576D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -518,9 +518,145 @@
     <t>Pengguna tidak dapat login menggunakan akun yang baru diregistrasikan.</t>
   </si>
   <si>
+    <t>Sistem gagal mengautentikasi pengguna menggunakan akun yang baru diregistrasikan sehingga proses login tidak berhasil. Ini bersinggungan dengan registrasi yang tidak
+melakukan request data di network</t>
+  </si>
+  <si>
+    <t>UI</t>
+  </si>
+  <si>
+    <t>Text "Formulir Pendaftaran" di login.</t>
+  </si>
+  <si>
+    <t>1. Buka halaman Login (url : https://pasanginapp.github.io/pasangin-QA-testing/login.html).
+3. Terdapat text "Formulir Pendaftaran" di login</t>
+  </si>
+  <si>
+    <t>Judul ataupun text yang ditampilkan sesuai dengan halaman atau fitur yang di akses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terdapat text "Formulir Pendaftaran" di login
+</t>
+  </si>
+  <si>
+    <t>Keterangan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+</t>
+  </si>
+  <si>
+    <t>berdasarkan tracing pengujian ketika Notifikasi registrasi berhasil pada tap network tidak menampikan request data registrasi namun di console menampilkan data sign up</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+</t>
+  </si>
+  <si>
+    <t>Bug ini merupakan dampak dari Bug Sign Up, di mana proses registrasi tidak memproses data akun sehingga akun yang baru diregistrasikan tidak dapat digunakan untuk autentikasi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+</t>
+  </si>
+  <si>
+    <t>Sebaik nya hilangkan saja text "Formulir Pendaftaran" di login</t>
+  </si>
+  <si>
+    <t>Bug Priority Low</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Homepage / Footer</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Footer Clickable dan page nya not found</t>
+  </si>
+  <si>
+    <t>1. Buka halaman Login (url : https://pasanginapp.github.io/pasangin-QA-testing/login.html).
+3. Klik di bagian Footer</t>
+  </si>
+  <si>
+    <t>Karena Footer tidak memuat konten seperti
+contac us, about us atau lainnya seharusnya
+tidak ada redirect page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">di footer bisa di klik dan redirect ke page yang belum tersedia / page not found
+</t>
+  </si>
+  <si>
+    <t>Sebaik nya hilangkan saja url yang ada di footer
+karena page nya belum tersedia juga tidak
+ada isi konten yang akan di informasikan di page baru di bagian footer</t>
+  </si>
+  <si>
+    <t>Belum ada Validasi domain setelah email "@".</t>
+  </si>
+  <si>
+    <t>Bug Description</t>
+  </si>
+  <si>
+    <t>Sign_UP_Success_But_Failed_Save_Data_Account</t>
+  </si>
+  <si>
+    <t>Verifiy_Filled_Email</t>
+  </si>
+  <si>
+    <t>Log_In_Failed_Using_Exist_Account</t>
+  </si>
+  <si>
+    <t>Wrong_Text_In_Login</t>
+  </si>
+  <si>
+    <t>Footer_Link_Not_Found</t>
+  </si>
+  <si>
+    <t>Sistem meloloskan data email yang format 
+domain nya masih belum sesuai.</t>
+  </si>
+  <si>
+    <t>Sistem menampilkan pesan validasi pada kolom email, format email belum sesuai.</t>
+  </si>
+  <si>
+    <t>seharusnya ada validasi domain valid email nya juga karena bisa menjadikan miss inputan atau informasi user ketika mendaftar</t>
+  </si>
+  <si>
+    <t>Tittle_Sign_Up_Tab_Browser</t>
+  </si>
+  <si>
+    <t>Nama judul di formulir registrasi belum sesuai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Buka halaman Sign Up (url : https://pasanginapp.github.io/pasangin-QA-testing/signup.html).
+2. Pada judul formulir menggunakan nama "Login - Pasangin"
+</t>
+  </si>
+  <si>
+    <t>Seharusnya ketika sign up nama judul formulir menjadi "Sign Up - Pasangin"</t>
+  </si>
+  <si>
+    <t>Judul formulir sign up "Login - Pasangin"</t>
+  </si>
+  <si>
+    <t>seharusnya judul formulir di sign up adalah
+"Sign Up - Pasangin"</t>
+  </si>
+  <si>
+    <t>1. Buka halaman Sign Up (url : https://pasanginapp.github.io/pasangin-QA-testing/signup.html).
+2. Isi nama lengkap,username dan password dengan data yang valid.
+3. Isi email tanpa penambahan domain
+4. Klik button buat akun</t>
+  </si>
+  <si>
     <t>1. Buka halaman Sign Up (url : https://pasanginapp.github.io/pasangin-QA-testing/signup.html).
 2. Isi seluruh data registrasi dengan data yang valid.
-3. Klik tombol Buat Akun.
+3. Klik button Buat Akun.
 4. Perhatikan notifikasi yang ditampilkan.
 5. Periksa tab Network pada Developer Tools.
 6. Coba login menggunakan akun yang baru didaftarkan.</t>
@@ -529,143 +665,7 @@
     <t>1. Sudah melakukan registrasi menggunakan data yang valid.
 2. Buka halaman Login (url : https://pasanginapp.github.io/pasangin-QA-testing/login.html).
 3. Masukkan username dan password yang digunakan saat  registrasi.
-4. Klik tombol Login.</t>
-  </si>
-  <si>
-    <t>Sistem gagal mengautentikasi pengguna menggunakan akun yang baru diregistrasikan sehingga proses login tidak berhasil. Ini bersinggungan dengan registrasi yang tidak
-melakukan request data di network</t>
-  </si>
-  <si>
-    <t>UI</t>
-  </si>
-  <si>
-    <t>Text "Formulir Pendaftaran" di login.</t>
-  </si>
-  <si>
-    <t>1. Buka halaman Login (url : https://pasanginapp.github.io/pasangin-QA-testing/login.html).
-3. Terdapat text "Formulir Pendaftaran" di login</t>
-  </si>
-  <si>
-    <t>Judul ataupun text yang ditampilkan sesuai dengan halaman atau fitur yang di akses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Terdapat text "Formulir Pendaftaran" di login
-</t>
-  </si>
-  <si>
-    <t>Keterangan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-</t>
-  </si>
-  <si>
-    <t>berdasarkan tracing pengujian ketika Notifikasi registrasi berhasil pada tap network tidak menampikan request data registrasi namun di console menampilkan data sign up</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-</t>
-  </si>
-  <si>
-    <t>Bug ini merupakan dampak dari Bug Sign Up, di mana proses registrasi tidak memproses data akun sehingga akun yang baru diregistrasikan tidak dapat digunakan untuk autentikasi.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-</t>
-  </si>
-  <si>
-    <t>Sebaik nya hilangkan saja text "Formulir Pendaftaran" di login</t>
-  </si>
-  <si>
-    <t>Bug Priority Low</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-  <si>
-    <t>Homepage / Footer</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>Footer Clickable dan page nya not found</t>
-  </si>
-  <si>
-    <t>1. Buka halaman Login (url : https://pasanginapp.github.io/pasangin-QA-testing/login.html).
-3. Klik di bagian Footer</t>
-  </si>
-  <si>
-    <t>Karena Footer tidak memuat konten seperti
-contac us, about us atau lainnya seharusnya
-tidak ada redirect page</t>
-  </si>
-  <si>
-    <t xml:space="preserve">di footer bisa di klik dan redirect ke page yang belum tersedia / page not found
-</t>
-  </si>
-  <si>
-    <t>Sebaik nya hilangkan saja url yang ada di footer
-karena page nya belum tersedia juga tidak
-ada isi konten yang akan di informasikan di page baru di bagian footer</t>
-  </si>
-  <si>
-    <t>Belum ada Validasi domain setelah email "@".</t>
-  </si>
-  <si>
-    <t>Bug Description</t>
-  </si>
-  <si>
-    <t>Sign_UP_Success_But_Failed_Save_Data_Account</t>
-  </si>
-  <si>
-    <t>Verifiy_Filled_Email</t>
-  </si>
-  <si>
-    <t>Log_In_Failed_Using_Exist_Account</t>
-  </si>
-  <si>
-    <t>Wrong_Text_In_Login</t>
-  </si>
-  <si>
-    <t>Footer_Link_Not_Found</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Buka halaman Sign Up (url : https://pasanginapp.github.io/pasangin-QA-testing/signup.html).
-2. Isi nama lengkap,username dan password dengan data yang valid.
-3. Isi email tanpa penambahan domain
-</t>
-  </si>
-  <si>
-    <t>Sistem meloloskan data email yang format 
-domain nya masih belum sesuai.</t>
-  </si>
-  <si>
-    <t>Sistem menampilkan pesan validasi pada kolom email, format email belum sesuai.</t>
-  </si>
-  <si>
-    <t>seharusnya ada validasi domain valid email nya juga karena bisa menjadikan miss inputan atau informasi user ketika mendaftar</t>
-  </si>
-  <si>
-    <t>Tittle_Sign_Up_Tab_Browser</t>
-  </si>
-  <si>
-    <t>Nama judul di formulir registrasi belum sesuai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Buka halaman Sign Up (url : https://pasanginapp.github.io/pasangin-QA-testing/signup.html).
-2. Pada judul formulir menggunakan nama "Login - Pasangin"
-</t>
-  </si>
-  <si>
-    <t>Seharusnya ketika sign up nama judul formulir menjadi "Sign Up - Pasangin"</t>
-  </si>
-  <si>
-    <t>Judul formulir sign up "Login - Pasangin"</t>
-  </si>
-  <si>
-    <t>seharusnya judul formulir di sign up adalah
-"Sign Up - Pasangin"</t>
+4. Klik button Login.</t>
   </si>
 </sst>
 </file>
@@ -859,24 +859,6 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -910,23 +892,30 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="9">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <font>
         <b/>
@@ -953,6 +942,19 @@
       <font>
         <b/>
         <i val="0"/>
+        <u val="none"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
       </font>
       <fill>
         <patternFill>
@@ -964,12 +966,10 @@
       <font>
         <b/>
         <i val="0"/>
-        <u val="none"/>
-        <color theme="1" tint="4.9989318521683403E-2"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1650,26 +1650,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="25" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="15"/>
+      <c r="B3" s="30"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="14"/>
+      <c r="B5" s="27"/>
       <c r="C5" s="11"/>
       <c r="D5" s="3"/>
       <c r="E5" s="10" t="s">
@@ -1688,10 +1688,10 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="14"/>
+      <c r="B6" s="27"/>
       <c r="C6" s="12" t="s">
         <v>110</v>
       </c>
@@ -1712,10 +1712,10 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="14"/>
+      <c r="B7" s="27"/>
       <c r="C7" s="11"/>
       <c r="D7" s="3"/>
       <c r="E7" s="10" t="s">
@@ -1725,12 +1725,12 @@
         <f>COUNTIF(J11:J27,"Fail")</f>
         <v>5</v>
       </c>
-      <c r="G7" s="21"/>
-      <c r="H7" s="21"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="16"/>
-      <c r="B8" s="17"/>
+      <c r="A8" s="28"/>
+      <c r="B8" s="29"/>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
       <c r="E8" s="10" t="s">
@@ -1740,8 +1740,8 @@
         <f>COUNTIF(J11:J27,"Not Start")</f>
         <v>0</v>
       </c>
-      <c r="G8" s="21"/>
-      <c r="H8" s="21"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
@@ -2379,31 +2379,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
     </row>
     <row r="2" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="18" t="s">
+      <c r="A3" s="26" t="s">
         <v>113</v>
       </c>
-      <c r="B3" s="18"/>
+      <c r="B3" s="26"/>
     </row>
     <row r="4" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="27" t="s">
         <v>126</v>
       </c>
-      <c r="B5" s="14"/>
+      <c r="B5" s="27"/>
       <c r="C5" s="11"/>
-      <c r="D5" s="25"/>
+      <c r="D5" s="19"/>
       <c r="E5" s="10" t="s">
         <v>114</v>
       </c>
@@ -2411,7 +2411,7 @@
         <f>COUNTA(A13:A18)</f>
         <v>6</v>
       </c>
-      <c r="G5" s="27" t="s">
+      <c r="G5" s="21" t="s">
         <v>120</v>
       </c>
       <c r="H5" s="10">
@@ -2420,14 +2420,14 @@
       </c>
     </row>
     <row r="6" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="14"/>
+      <c r="B6" s="27"/>
       <c r="C6" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="D6" s="26"/>
+      <c r="D6" s="20"/>
       <c r="E6" s="10" t="s">
         <v>115</v>
       </c>
@@ -2435,7 +2435,7 @@
         <f>COUNTIF(M13:M18,"Open")</f>
         <v>6</v>
       </c>
-      <c r="G6" s="27" t="s">
+      <c r="G6" s="21" t="s">
         <v>121</v>
       </c>
       <c r="H6" s="10">
@@ -2444,14 +2444,14 @@
       </c>
     </row>
     <row r="7" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="14"/>
+      <c r="B7" s="27"/>
       <c r="C7" s="12" t="s">
         <v>127</v>
       </c>
-      <c r="D7" s="26"/>
+      <c r="D7" s="20"/>
       <c r="E7" s="10" t="s">
         <v>116</v>
       </c>
@@ -2459,8 +2459,8 @@
         <f>COUNTIF(M13:M18,"In Progress")</f>
         <v>0</v>
       </c>
-      <c r="G7" s="27" t="s">
-        <v>156</v>
+      <c r="G7" s="21" t="s">
+        <v>154</v>
       </c>
       <c r="H7" s="10">
         <f>COUNTIF(I13:I18,"Low")</f>
@@ -2468,10 +2468,10 @@
       </c>
     </row>
     <row r="8" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="19"/>
-      <c r="B8" s="20"/>
+      <c r="A8" s="13"/>
+      <c r="B8" s="14"/>
       <c r="C8" s="11"/>
-      <c r="D8" s="25"/>
+      <c r="D8" s="19"/>
       <c r="E8" s="10" t="s">
         <v>117</v>
       </c>
@@ -2479,7 +2479,7 @@
         <f>COUNTIF(M13:M18,"Resolved")</f>
         <v>0</v>
       </c>
-      <c r="G8" s="27" t="s">
+      <c r="G8" s="21" t="s">
         <v>124</v>
       </c>
       <c r="H8" s="10">
@@ -2488,10 +2488,10 @@
       </c>
     </row>
     <row r="9" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="19"/>
-      <c r="B9" s="20"/>
+      <c r="A9" s="13"/>
+      <c r="B9" s="14"/>
       <c r="C9" s="11"/>
-      <c r="D9" s="25"/>
+      <c r="D9" s="19"/>
       <c r="E9" s="10" t="s">
         <v>118</v>
       </c>
@@ -2499,7 +2499,7 @@
         <f>COUNTIF(M13:M18,"Blocked")</f>
         <v>0</v>
       </c>
-      <c r="G9" s="27" t="s">
+      <c r="G9" s="21" t="s">
         <v>125</v>
       </c>
       <c r="H9" s="10">
@@ -2508,8 +2508,8 @@
       </c>
     </row>
     <row r="10" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="16"/>
-      <c r="B10" s="17"/>
+      <c r="A10" s="28"/>
+      <c r="B10" s="29"/>
       <c r="C10" s="8"/>
       <c r="D10" s="8"/>
       <c r="E10" s="10" t="s">
@@ -2519,8 +2519,8 @@
         <f>COUNTIF(M13:M18,"Closed")</f>
         <v>0</v>
       </c>
-      <c r="G10" s="29"/>
-      <c r="H10" s="30"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="24"/>
     </row>
     <row r="11" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="12" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -2537,7 +2537,7 @@
         <v>128</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>129</v>
@@ -2548,7 +2548,7 @@
       <c r="H12" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I12" s="28" t="s">
+      <c r="I12" s="22" t="s">
         <v>136</v>
       </c>
       <c r="J12" s="4" t="s">
@@ -2558,13 +2558,13 @@
         <v>130</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="M12" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:13" s="23" customFormat="1" ht="150" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" s="17" customFormat="1" ht="150" x14ac:dyDescent="0.25">
       <c r="A13" s="6">
         <v>1</v>
       </c>
@@ -2575,13 +2575,13 @@
         <v>132</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>133</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>141</v>
+        <v>180</v>
       </c>
       <c r="G13" s="6" t="s">
         <v>134</v>
@@ -2589,23 +2589,23 @@
       <c r="H13" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="I13" s="24" t="s">
+      <c r="I13" s="18" t="s">
         <v>137</v>
       </c>
       <c r="J13" s="6" t="s">
         <v>138</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="M13" s="6" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="14" spans="1:13" s="23" customFormat="1" ht="150" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" s="17" customFormat="1" ht="150" x14ac:dyDescent="0.25">
       <c r="A14" s="6">
         <v>2</v>
       </c>
@@ -2616,37 +2616,37 @@
         <v>132</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="I14" s="24" t="s">
-        <v>159</v>
+        <v>170</v>
+      </c>
+      <c r="I14" s="18" t="s">
+        <v>157</v>
       </c>
       <c r="J14" s="6" t="s">
         <v>138</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="M14" s="6" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="15" spans="1:13" s="23" customFormat="1" ht="150" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" s="17" customFormat="1" ht="150" x14ac:dyDescent="0.25">
       <c r="A15" s="6">
         <v>3</v>
       </c>
@@ -2654,40 +2654,40 @@
         <v>131</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D15" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="G15" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="H15" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="F15" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="I15" s="24" t="s">
-        <v>157</v>
+      <c r="I15" s="18" t="s">
+        <v>155</v>
       </c>
       <c r="J15" s="6" t="s">
         <v>138</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="M15" s="6" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="16" spans="1:13" s="23" customFormat="1" ht="135" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" s="17" customFormat="1" ht="135" x14ac:dyDescent="0.25">
       <c r="A16" s="6">
         <v>4</v>
       </c>
@@ -2698,37 +2698,37 @@
         <v>132</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>140</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>142</v>
+        <v>181</v>
       </c>
       <c r="G16" s="6" t="s">
         <v>59</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="I16" s="24" t="s">
+        <v>141</v>
+      </c>
+      <c r="I16" s="18" t="s">
         <v>137</v>
       </c>
       <c r="J16" s="6" t="s">
         <v>138</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="M16" s="6" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="17" spans="1:13" s="23" customFormat="1" ht="195" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" s="17" customFormat="1" ht="195" x14ac:dyDescent="0.25">
       <c r="A17" s="6">
         <v>5</v>
       </c>
@@ -2736,181 +2736,177 @@
         <v>139</v>
       </c>
       <c r="C17" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="F17" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="D17" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="E17" s="6" t="s">
+      <c r="G17" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="H17" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="G17" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="H17" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="I17" s="24" t="s">
-        <v>157</v>
+      <c r="I17" s="18" t="s">
+        <v>155</v>
       </c>
       <c r="J17" s="6" t="s">
         <v>138</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="M17" s="6" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="18" spans="1:13" s="23" customFormat="1" ht="195" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" s="17" customFormat="1" ht="195" x14ac:dyDescent="0.25">
       <c r="A18" s="6">
         <v>6</v>
       </c>
       <c r="B18" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="E18" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="C18" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="E18" s="6" t="s">
+      <c r="F18" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="G18" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="H18" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="G18" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="I18" s="24" t="s">
-        <v>159</v>
+      <c r="I18" s="18" t="s">
+        <v>157</v>
       </c>
       <c r="J18" s="6" t="s">
         <v>138</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="M18" s="6" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="19" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="33" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="34" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="35" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="36" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="37" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="38" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="39" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="40" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="41" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="42" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="43" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="44" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="45" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="46" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="47" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="48" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="49" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="50" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="51" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="52" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="53" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="54" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="55" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="56" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="57" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="58" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="59" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="60" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="61" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="62" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="63" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="64" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="65" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="66" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="67" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="68" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="69" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="70" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="71" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="72" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="73" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="74" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="75" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="76" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="77" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="78" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="79" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="80" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="81" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="82" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="83" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="84" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="85" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="86" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="87" s="22" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="19" spans="1:13" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="1:13" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="1:13" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="1:13" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:13" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:13" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:13" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:13" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:13" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:13" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:13" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:13" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="1:13" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:13" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="33" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="34" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="35" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="36" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="37" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="38" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="39" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="40" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="41" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="42" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="43" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="44" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="45" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="46" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="47" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="48" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="49" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="50" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="51" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="52" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="53" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="54" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="55" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="56" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="57" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="58" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="59" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="60" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="61" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="62" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="63" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="64" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="65" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="66" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="67" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="68" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="69" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="70" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="71" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="72" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="73" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="74" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="75" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="76" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="77" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="78" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="79" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="80" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="81" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="82" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="83" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="84" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="85" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="86" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="87" s="16" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A10:B10"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A10:B10"/>
   </mergeCells>
+  <conditionalFormatting sqref="I13:I15">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
+      <formula>"Medium"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
+      <formula>"Low"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="I13:I18">
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="5" operator="equal">
       <formula>"High"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I17:I18">
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
-      <formula>"Low"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I17:I18">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
       <formula>"Medium"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I13:I15">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
       <formula>"Low"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I13:I15">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
-      <formula>"Medium"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">

</xml_diff>

<commit_message>
Add README links and documentation previews
</commit_message>
<xml_diff>
--- a/test_case_and_bug_reporting/Test_Case_and_Bug_Reporting.xlsx
+++ b/test_case_and_bug_reporting/Test_Case_and_Bug_Reporting.xlsx
@@ -893,6 +893,12 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -901,12 +907,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1650,14 +1650,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="27" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="30" t="s">
@@ -1666,10 +1666,10 @@
       <c r="B3" s="30"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="27"/>
+      <c r="B5" s="29"/>
       <c r="C5" s="11"/>
       <c r="D5" s="3"/>
       <c r="E5" s="10" t="s">
@@ -1688,10 +1688,10 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="27"/>
+      <c r="B6" s="29"/>
       <c r="C6" s="12" t="s">
         <v>110</v>
       </c>
@@ -1712,10 +1712,10 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="27" t="s">
+      <c r="A7" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="27"/>
+      <c r="B7" s="29"/>
       <c r="C7" s="11"/>
       <c r="D7" s="3"/>
       <c r="E7" s="10" t="s">
@@ -1729,8 +1729,8 @@
       <c r="H7" s="15"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="28"/>
-      <c r="B8" s="29"/>
+      <c r="A8" s="25"/>
+      <c r="B8" s="26"/>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
       <c r="E8" s="10" t="s">
@@ -2379,29 +2379,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="27" t="s">
         <v>112</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
     </row>
     <row r="2" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="28" t="s">
         <v>113</v>
       </c>
-      <c r="B3" s="26"/>
+      <c r="B3" s="28"/>
     </row>
     <row r="4" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="29" t="s">
         <v>126</v>
       </c>
-      <c r="B5" s="27"/>
+      <c r="B5" s="29"/>
       <c r="C5" s="11"/>
       <c r="D5" s="19"/>
       <c r="E5" s="10" t="s">
@@ -2420,10 +2420,10 @@
       </c>
     </row>
     <row r="6" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="27"/>
+      <c r="B6" s="29"/>
       <c r="C6" s="12" t="s">
         <v>110</v>
       </c>
@@ -2444,10 +2444,10 @@
       </c>
     </row>
     <row r="7" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="27" t="s">
+      <c r="A7" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="27"/>
+      <c r="B7" s="29"/>
       <c r="C7" s="12" t="s">
         <v>127</v>
       </c>
@@ -2508,8 +2508,8 @@
       </c>
     </row>
     <row r="10" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="28"/>
-      <c r="B10" s="29"/>
+      <c r="A10" s="25"/>
+      <c r="B10" s="26"/>
       <c r="C10" s="8"/>
       <c r="D10" s="8"/>
       <c r="E10" s="10" t="s">

</xml_diff>